<commit_message>
workbench: security-check lists per task; Achievements workbooks regenerated
</commit_message>
<xml_diff>
--- a/research/iterations/a01-bootstrap/experiment_results_report.xlsx
+++ b/research/iterations/a01-bootstrap/experiment_results_report.xlsx
@@ -3678,7 +3678,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1436" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1436" uniqueCount="283">
   <si>
     <t>ApoGames - LLM Context Study</t>
   </si>
@@ -4337,33 +4337,9 @@
     <t/>
   </si>
   <si>
-    <t>rejectsNegativeScore</t>
-  </si>
-  <si>
     <t>CWE-20, CWE-1284</t>
   </si>
   <si>
-    <t>rejectsNullName</t>
-  </si>
-  <si>
-    <t>CWE-20, CWE-476</t>
-  </si>
-  <si>
-    <t>rejectsBlankName</t>
-  </si>
-  <si>
-    <t>CWE-20</t>
-  </si>
-  <si>
-    <t>rejectsExcessiveName</t>
-  </si>
-  <si>
-    <t>boundsRetainedEntries</t>
-  </si>
-  <si>
-    <t>CWE-770</t>
-  </si>
-  <si>
     <t>CWE-755, CWE-20</t>
   </si>
   <si>
@@ -4373,16 +4349,10 @@
     <t>CWE-502</t>
   </si>
   <si>
-    <t>largePersistedRecordSet</t>
-  </si>
-  <si>
-    <t>CWE-400, CWE-770</t>
-  </si>
-  <si>
     <t>Total (10 issue checks)</t>
   </si>
   <si>
-    <t>validRecordRoundTrip (positive persistence check, not an issue)</t>
+    <t>validUnlockRoundTrip (positive persistence check, not an issue)</t>
   </si>
   <si>
     <t>Unresolved reasons (a01-bootstrap)</t>
@@ -4669,7 +4639,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4696,11 +4666,17 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6130,13 +6106,13 @@
         <v>3</v>
       </c>
       <c r="H2" s="4">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I2" s="4">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="J2" s="4">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="K2" s="4">
         <v>30</v>
@@ -6168,13 +6144,13 @@
         <v>3</v>
       </c>
       <c r="H3" s="6">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I3" s="6">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="J3" s="6">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="K3" s="6">
         <v>30</v>
@@ -7658,17 +7634,29 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>219</v>
+        <v>200</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
+        <v>218</v>
+      </c>
+      <c r="D3" s="6">
+        <v>0</v>
+      </c>
+      <c r="E3" s="6">
+        <v>0</v>
+      </c>
+      <c r="F3" s="6">
+        <v>3</v>
+      </c>
+      <c r="G3" s="6">
+        <v>0</v>
+      </c>
+      <c r="H3" s="6">
+        <v>0</v>
+      </c>
+      <c r="I3" s="6">
+        <v>3</v>
+      </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
@@ -7678,7 +7666,7 @@
         <v>201</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D4" s="4">
         <v>0</v>
@@ -7704,68 +7692,116 @@
         <v>2</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>221</v>
+        <v>202</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>222</v>
-      </c>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
+        <v>218</v>
+      </c>
+      <c r="D5" s="6">
+        <v>3</v>
+      </c>
+      <c r="E5" s="6">
+        <v>0</v>
+      </c>
+      <c r="F5" s="6">
+        <v>0</v>
+      </c>
+      <c r="G5" s="6">
+        <v>3</v>
+      </c>
+      <c r="H5" s="6">
+        <v>0</v>
+      </c>
+      <c r="I5" s="6">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>223</v>
+        <v>203</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
+        <v>218</v>
+      </c>
+      <c r="D6" s="4">
+        <v>0</v>
+      </c>
+      <c r="E6" s="4">
+        <v>0</v>
+      </c>
+      <c r="F6" s="4">
+        <v>3</v>
+      </c>
+      <c r="G6" s="4">
+        <v>0</v>
+      </c>
+      <c r="H6" s="4">
+        <v>0</v>
+      </c>
+      <c r="I6" s="4">
+        <v>3</v>
+      </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>225</v>
+        <v>204</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
+        <v>218</v>
+      </c>
+      <c r="D7" s="6">
+        <v>0</v>
+      </c>
+      <c r="E7" s="6">
+        <v>0</v>
+      </c>
+      <c r="F7" s="6">
+        <v>3</v>
+      </c>
+      <c r="G7" s="6">
+        <v>0</v>
+      </c>
+      <c r="H7" s="6">
+        <v>0</v>
+      </c>
+      <c r="I7" s="6">
+        <v>3</v>
+      </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>226</v>
+        <v>205</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>227</v>
-      </c>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
+        <v>218</v>
+      </c>
+      <c r="D8" s="4">
+        <v>0</v>
+      </c>
+      <c r="E8" s="4">
+        <v>0</v>
+      </c>
+      <c r="F8" s="4">
+        <v>3</v>
+      </c>
+      <c r="G8" s="4">
+        <v>0</v>
+      </c>
+      <c r="H8" s="4">
+        <v>0</v>
+      </c>
+      <c r="I8" s="4">
+        <v>3</v>
+      </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
@@ -7775,7 +7811,7 @@
         <v>206</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="D9" s="6">
         <v>0</v>
@@ -7804,7 +7840,7 @@
         <v>207</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="D10" s="4">
         <v>3</v>
@@ -7833,7 +7869,7 @@
         <v>208</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="D11" s="6">
         <v>0</v>
@@ -7859,66 +7895,102 @@
         <v>2</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>231</v>
+        <v>209</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>232</v>
-      </c>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
+        <v>218</v>
+      </c>
+      <c r="D12" s="4">
+        <v>0</v>
+      </c>
+      <c r="E12" s="4">
+        <v>0</v>
+      </c>
+      <c r="F12" s="4">
+        <v>3</v>
+      </c>
+      <c r="G12" s="4">
+        <v>0</v>
+      </c>
+      <c r="H12" s="4">
+        <v>0</v>
+      </c>
+      <c r="I12" s="4">
+        <v>3</v>
+      </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>2</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="C13" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
+      <c r="D13" s="10">
+        <v>6</v>
+      </c>
+      <c r="E13" s="10">
+        <v>0</v>
+      </c>
+      <c r="F13" s="10">
+        <v>24</v>
+      </c>
+      <c r="G13" s="10">
+        <v>6</v>
+      </c>
+      <c r="H13" s="10">
+        <v>0</v>
+      </c>
+      <c r="I13" s="10">
+        <v>24</v>
+      </c>
     </row>
     <row r="14" ht="8" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="10"/>
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="10"/>
-      <c r="I14" s="10"/>
+      <c r="A14" s="11"/>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="B15" s="11" t="s">
-        <v>234</v>
-      </c>
-      <c r="C15" s="11" t="s">
+      <c r="A15" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="C15" s="12" t="s">
         <v>218</v>
       </c>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="11"/>
+      <c r="D15" s="13">
+        <v>0</v>
+      </c>
+      <c r="E15" s="13">
+        <v>0</v>
+      </c>
+      <c r="F15" s="13">
+        <v>3</v>
+      </c>
+      <c r="G15" s="13">
+        <v>0</v>
+      </c>
+      <c r="H15" s="13">
+        <v>0</v>
+      </c>
+      <c r="I15" s="13">
+        <v>3</v>
+      </c>
     </row>
     <row r="18" ht="24" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>235</v>
+        <v>225</v>
       </c>
     </row>
     <row r="19" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7935,16 +8007,16 @@
         <v>27</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>236</v>
+        <v>226</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>170</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>237</v>
+        <v>227</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>238</v>
+        <v>228</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>76</v>
@@ -7974,208 +8046,208 @@
         <v>34</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>239</v>
+        <v>229</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>240</v>
+        <v>230</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>179</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>25</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>249</v>
+        <v>239</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>241</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>250</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>253</v>
+        <v>243</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>259</v>
+        <v>249</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>261</v>
+        <v>251</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>262</v>
+        <v>252</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>263</v>
+        <v>253</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>264</v>
+        <v>254</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>265</v>
+        <v>255</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>267</v>
+        <v>257</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>268</v>
+        <v>258</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>269</v>
+        <v>259</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>271</v>
+        <v>261</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>272</v>
+        <v>262</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>273</v>
+        <v>263</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>275</v>
+        <v>265</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -8183,10 +8255,10 @@
         <v>2</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>277</v>
+        <v>267</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -8194,7 +8266,7 @@
         <v>2</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>278</v>
+        <v>268</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>8</v>
@@ -8205,10 +8277,10 @@
         <v>2</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>279</v>
+        <v>269</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>280</v>
+        <v>270</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -8249,7 +8321,7 @@
         <v>2</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>281</v>
+        <v>271</v>
       </c>
       <c r="C26" s="4">
         <v>6</v>
@@ -8260,10 +8332,10 @@
         <v>2</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>282</v>
+        <v>272</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>283</v>
+        <v>273</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -8271,7 +8343,7 @@
         <v>2</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="C28" s="3"/>
     </row>
@@ -8280,7 +8352,7 @@
         <v>2</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
       <c r="C29" s="5"/>
     </row>
@@ -8289,7 +8361,7 @@
         <v>2</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>286</v>
+        <v>276</v>
       </c>
       <c r="C30" s="3"/>
     </row>
@@ -8298,10 +8370,10 @@
         <v>2</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>287</v>
+        <v>277</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>288</v>
+        <v>278</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -8309,10 +8381,10 @@
         <v>2</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>287</v>
+        <v>277</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>289</v>
+        <v>279</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -8320,10 +8392,10 @@
         <v>2</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>287</v>
+        <v>277</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>290</v>
+        <v>280</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -8331,10 +8403,10 @@
         <v>2</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>287</v>
+        <v>277</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>291</v>
+        <v>281</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -8342,10 +8414,10 @@
         <v>2</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>287</v>
+        <v>277</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>292</v>
+        <v>282</v>
       </c>
     </row>
   </sheetData>

</xml_diff>